<commit_message>
docs: correct figure evidence and unify citation navigation
Replace overview and segmentation captures, use both pages of one authentic report, distinguish independent cancellation records, add alternative text and tagged PDF, and package cited companion materials. Preserve source-specific test results and uncollected study status.
</commit_message>
<xml_diff>
--- a/current-software-2026-10-27/Evaluation_Materials/Windows_Manual_Acceptance_Reviewed.xlsx
+++ b/current-software-2026-10-27/Evaluation_Materials/Windows_Manual_Acceptance_Reviewed.xlsx
@@ -922,7 +922,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Real operation progresses228/400; cancellation is acknowledged and displayed record79 is retained.</t>
+          <t>Independent observations: classification progress228/400 withSession record79; separate cancellation acknowledgement withretained classification record78 andSegmentation selected. No continuous before/after sequence established.</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
@@ -937,7 +937,7 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>Record database/history outcome and close-while-busy cleanup; transient Cancelling screenshot is not required.</t>
+          <t>Record one continuous cancellation and history outcome; separately record close-while-busy cleanup. No transient Cancelling screenshot is required.</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr"/>

</xml_diff>